<commit_message>
pipeline: arnona idx 9, 09.07.2026
</commit_message>
<xml_diff>
--- a/reports/דוח נכסים חשודים 09.07.2026.xlsx
+++ b/reports/דוח נכסים חשודים 09.07.2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="דוח עסקים חשודים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="דוח נכסים חשודים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,10 +26,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -38,12 +45,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD700"/>
-        <bgColor rgb="00FFD700"/>
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -51,14 +64,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,18 +451,18 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>שם העסק</t>
@@ -492,51 +514,51 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>גרין נט מחזור וטיפול בפסולת בע"מ</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>מחזור וטיפול בפסולת</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>שדה תעופה עטרות 26</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>מוסך דיזל עטרות ירושלים בע"מ</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>מוסך (רכב)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>שדה תעופה עטרות 35</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>שדה תעופה עטרות 26</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>שדה תעופה עטרות 35</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה — ריצת DEMO</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>https://www.dunsguide.co.il/C672e66e79d35ae7af7a63104e8d7a17f_%D7%97%D7%91%D7%A8%D7%95%D7%AA_%D7%94%D7%99%D7%99%D7%98%D7%A7_%D7%95%D7%9E%D7%99%D7%97%D7%A9%D7%95%D7%91/%D7%92%D7%A8%D7%99%D7%9F_%D7%A0%D7%98_%D7%9E%D7%97%D7%96%D7%95%D7%A8_%D7%95%D7%98%D7%99%D7%A4%D7%95%D7%9C_%D7%91%D7%A4%D7%A1%D7%95%D7%9C%D7%AA</t>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/8579530/28275</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pipeline: arnona idx 19, 09.07.2026
DEMO run — processed indices 9–18 (streets: שדה תעופה עטרות, אבא אבן).
Found 1 verified suspicious business: מסגריית הפתרון at אבא אבן 1, ירושלים.
</commit_message>
<xml_diff>
--- a/reports/דוח נכסים חשודים 09.07.2026.xlsx
+++ b/reports/דוח נכסים חשודים 09.07.2026.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,17 +26,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -45,18 +38,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
-        <bgColor rgb="00FFF3CD"/>
+        <fgColor rgb="00FFD700"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -64,23 +50,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -450,19 +427,19 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>שם העסק</t>
@@ -514,51 +491,51 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>מוסך דיזל עטרות ירושלים בע"מ</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>מוסך (רכב)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>שדה תעופה עטרות 35</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>מסגריית הפתרון</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>מסגרייה — מסגרות ברזל ושערים חשמליים</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>אבא אבן 1, ירושלים</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>שדה תעופה עטרות 35</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>אבא אבן 1, ירושלים</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה — ריצת DEMO</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/8579530/28275</t>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80342103/49680</t>
         </is>
       </c>
     </row>

</xml_diff>